<commit_message>
Improve transcription accuracy and suppress hallucinations
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/evaluation/EVALUACION-VOZLARGA-10-10.xlsx
+++ b/evaluation/EVALUACION-VOZLARGA-10-10.xlsx
@@ -196,7 +196,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Faltan los 5 audios y sus guiones. Whisper Small es multilingüe; no implica cumplir el umbral.</t>
+          <t xml:space="preserve">Faltan los 5 audios y sus guiones. Whisper Large v3 Turbo es multilingüe; no implica cumplir el umbral.</t>
         </is>
       </c>
     </row>
@@ -260,7 +260,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pipeline completo: 7200 s procesados en 1261 s, 9/9 bloques. No usa Small ni RX 5600 XT, por tanto no certifica producto final.</t>
+          <t xml:space="preserve">Pipeline completo: 7200 s procesados en 1261 s, 9/9 bloques. No usa Large v3 Turbo ni RX 5600 XT, por tanto no certifica producto final.</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">APROBADO PARA FLUJO, NO PARA SMALL/GPU</t>
+          <t xml:space="preserve">APROBADO PARA FLUJO, NO PARA TURBO/GPU</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FALLÓ; mitigado: VAD solo Vulkan y off por defecto</t>
+          <t xml:space="preserve">FALLÓ; mitigado: VAD solo Vulkan; el respaldo CPU lo omite</t>
         </is>
       </c>
     </row>

</xml_diff>